<commit_message>
Etapa 8-9: verificador de integridade + graficos Chart.js + simulador interativo no HTML
</commit_message>
<xml_diff>
--- a/dist/modelo.xlsx
+++ b/dist/modelo.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\w.marreiro\Desktop\PRODUCT MANAGEMENT\SAAS - BILLING BUSINESS MODEL\irricontrol-one-receita\dist\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{5BD78747-4186-43B7-B4BA-9120311FFF97}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{9A6B9659-FDD2-49A1-B9E7-9CFA5E9728C4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1152" yWindow="1152" windowWidth="17280" windowHeight="8880" xr2:uid="{DDABA7ED-A613-4BDC-932A-F4350995F9A6}"/>
+    <workbookView xWindow="1152" yWindow="1152" windowWidth="17280" windowHeight="8880" xr2:uid="{D22A4592-A624-4176-A1AC-0532DA1B934C}"/>
   </bookViews>
   <sheets>
     <sheet name="Receita Escondida" sheetId="8" r:id="rId1"/>
@@ -833,7 +833,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F06BCC97-A846-4B2C-9EAE-EFA2811AF5C4}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{77A6BC28-E347-4B42-ADB1-332EF98ADCED}">
   <dimension ref="A1:I6"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
@@ -1028,7 +1028,7 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A1DFD1E8-F8D0-4970-95BC-80F31E9FB2D7}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{36C57AFA-7231-47EB-BDF7-59C5F23DE953}">
   <dimension ref="A1:P16"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
@@ -1856,7 +1856,7 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EE17FC57-2961-443F-9C07-CF4270409632}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B6DEF338-C407-4CC7-9F7C-B7EDD0C118AF}">
   <dimension ref="A1:E11"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
@@ -2059,7 +2059,7 @@
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{308A39BF-FFBB-46AE-9637-E8B6113BD1C2}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{938C1E0D-9C19-4C71-B822-BC7949DC9D10}">
   <dimension ref="A1:C42"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
@@ -2535,7 +2535,7 @@
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2BF1113E-846D-45FD-A4A7-A42EEFABD0BA}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B141AFE5-B7B8-4317-B3FC-9A9AE8886C9F}">
   <dimension ref="A1:B8"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
@@ -2613,7 +2613,7 @@
 </file>
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D1097B08-434D-4699-816E-0CE45EBD8246}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{781BD633-0532-46F8-AB61-E47D0A3BFBAD}">
   <dimension ref="A1:B24"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
@@ -2819,7 +2819,7 @@
 </file>
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4EC9D954-4B91-42EF-A7C8-C5D30816A73C}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D72A9D5C-27BE-4279-9322-10D3885C563B}">
   <dimension ref="A1:B22"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
@@ -3009,7 +3009,7 @@
 </file>
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4B94F040-BD6A-476E-91FA-28F79C93E684}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AD300348-C963-45E1-B61E-2D95C7F779CA}">
   <dimension ref="A1"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData/>

</xml_diff>

<commit_message>
feat: consolidar pipeline de receita SaaS
</commit_message>
<xml_diff>
--- a/dist/modelo.xlsx
+++ b/dist/modelo.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\w.marreiro\Desktop\PRODUCT MANAGEMENT\SAAS - BILLING BUSINESS MODEL\irricontrol-one-receita\dist\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{9A6B9659-FDD2-49A1-B9E7-9CFA5E9728C4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{E4802E60-0136-49EC-A03C-0072AF993FCD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1152" yWindow="1152" windowWidth="17280" windowHeight="8880" xr2:uid="{D22A4592-A624-4176-A1AC-0532DA1B934C}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{75876D50-A835-4BA3-BA65-2414C1CD2AE3}"/>
   </bookViews>
   <sheets>
     <sheet name="Receita Escondida" sheetId="8" r:id="rId1"/>
@@ -46,7 +46,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="164" uniqueCount="131">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="138" uniqueCount="103">
   <si>
     <t>Metrica</t>
   </si>
@@ -126,6 +126,12 @@
     <t>anuidadeRef</t>
   </si>
   <si>
+    <t>anuidadeIrripump</t>
+  </si>
+  <si>
+    <t>anuidadeMedidorNivel</t>
+  </si>
+  <si>
     <t>precoTabelaSaaS</t>
   </si>
   <si>
@@ -198,7 +204,10 @@
     <t>pivos</t>
   </si>
   <si>
-    <t>{"total":3926,"testeDemo":79,"efetivos":3847}</t>
+    <t>{"total":3926,"testeDemo":79,"efetivos":3847,"smartRainMigrados":43}</t>
+  </si>
+  <si>
+    <t>hoseReels</t>
   </si>
   <si>
     <t>irripump</t>
@@ -207,145 +216,52 @@
     <t>medidorNivel</t>
   </si>
   <si>
+    <t>offGridRainGauges</t>
+  </si>
+  <si>
     <t>fazendas</t>
   </si>
   <si>
+    <t>fazendasUsandoAPI</t>
+  </si>
+  <si>
     <t>usuariosAtivos</t>
   </si>
   <si>
     <t>pontosPagantes</t>
   </si>
   <si>
-    <t>Mes</t>
-  </si>
-  <si>
-    <t>2023-04</t>
-  </si>
-  <si>
-    <t>Charge</t>
-  </si>
-  <si>
-    <t>Invoice</t>
-  </si>
-  <si>
-    <t>2023-05</t>
-  </si>
-  <si>
-    <t>2023-06</t>
-  </si>
-  <si>
-    <t>2023-07</t>
-  </si>
-  <si>
-    <t>2023-08</t>
-  </si>
-  <si>
-    <t>2023-09</t>
-  </si>
-  <si>
-    <t>2023-10</t>
-  </si>
-  <si>
-    <t>2023-11</t>
-  </si>
-  <si>
-    <t>2023-12</t>
-  </si>
-  <si>
-    <t>2024-01</t>
-  </si>
-  <si>
-    <t>2024-02</t>
-  </si>
-  <si>
-    <t>2024-03</t>
-  </si>
-  <si>
-    <t>2024-04</t>
-  </si>
-  <si>
-    <t>2024-05</t>
-  </si>
-  <si>
-    <t>2024-06</t>
-  </si>
-  <si>
-    <t>2024-07</t>
-  </si>
-  <si>
-    <t>2024-08</t>
-  </si>
-  <si>
-    <t>2024-09</t>
-  </si>
-  <si>
-    <t>2024-10</t>
-  </si>
-  <si>
-    <t>2024-11</t>
-  </si>
-  <si>
-    <t>2024-12</t>
-  </si>
-  <si>
-    <t>2025-01</t>
-  </si>
-  <si>
-    <t>2025-02</t>
-  </si>
-  <si>
-    <t>2025-03</t>
-  </si>
-  <si>
-    <t>2025-04</t>
-  </si>
-  <si>
-    <t>2025-05</t>
-  </si>
-  <si>
-    <t>2025-06</t>
-  </si>
-  <si>
-    <t>2025-07</t>
-  </si>
-  <si>
-    <t>2025-08</t>
-  </si>
-  <si>
-    <t>2025-09</t>
-  </si>
-  <si>
-    <t>2025-10</t>
-  </si>
-  <si>
-    <t>2025-11</t>
-  </si>
-  <si>
-    <t>2025-12</t>
-  </si>
-  <si>
-    <t>2026-01</t>
-  </si>
-  <si>
-    <t>2026-02</t>
-  </si>
-  <si>
-    <t>2026-03</t>
-  </si>
-  <si>
-    <t>2026-04</t>
-  </si>
-  <si>
-    <t>2026-05</t>
-  </si>
-  <si>
-    <t>2026-06</t>
-  </si>
-  <si>
-    <t>2026-07</t>
-  </si>
-  <si>
-    <t>2026-08</t>
+    <t>IsReadOnly</t>
+  </si>
+  <si>
+    <t>Nao</t>
+  </si>
+  <si>
+    <t>IsFixedSize</t>
+  </si>
+  <si>
+    <t>IsSynchronized</t>
+  </si>
+  <si>
+    <t>Keys</t>
+  </si>
+  <si>
+    <t>2024-05 2026-03 2026-08 2025-08 2024-06 2026-01 2025-02 2025-11 2024-04 2026-02 2024-11 2024-02 2025-09 2024-01 2025-06 2024-03 2026-06 2023-04 2024-12 2025-04 2025-10 2025-01 2023-06 2026-04 2024-10 2026-07 2025-07 2024-09 2024-08 2025-05 2023-05 2023-08 2025-03 2026-05 2025-12 2024-07</t>
+  </si>
+  <si>
+    <t>Values</t>
+  </si>
+  <si>
+    <t xml:space="preserve">                                   </t>
+  </si>
+  <si>
+    <t>SyncRoot</t>
+  </si>
+  <si>
+    <t>System.Object</t>
+  </si>
+  <si>
+    <t>Count</t>
   </si>
   <si>
     <t>Tipo</t>
@@ -833,7 +749,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{77A6BC28-E347-4B42-ADB1-332EF98ADCED}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F4EF9C60-B8E9-46AD-9765-6F7A7FF515EE}">
   <dimension ref="A1:I6"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
@@ -850,31 +766,31 @@
   <sheetData>
     <row r="1" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A1" s="4" t="s">
-        <v>112</v>
+        <v>84</v>
       </c>
       <c r="B1" s="4" t="s">
-        <v>114</v>
+        <v>86</v>
       </c>
       <c r="C1" s="4" t="s">
-        <v>123</v>
+        <v>95</v>
       </c>
       <c r="D1" s="4" t="s">
-        <v>116</v>
+        <v>88</v>
       </c>
       <c r="E1" s="4" t="s">
-        <v>115</v>
+        <v>87</v>
       </c>
       <c r="F1" s="4" t="s">
-        <v>117</v>
+        <v>89</v>
       </c>
       <c r="G1" s="4" t="s">
-        <v>129</v>
+        <v>101</v>
       </c>
       <c r="H1" s="4" t="s">
-        <v>121</v>
+        <v>93</v>
       </c>
       <c r="I1" s="4" t="s">
-        <v>130</v>
+        <v>102</v>
       </c>
     </row>
     <row r="2" spans="1:9" x14ac:dyDescent="0.3">
@@ -1028,7 +944,7 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{36C57AFA-7231-47EB-BDF7-59C5F23DE953}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C48F06A4-5C61-4C27-B662-EA757A57C3E4}">
   <dimension ref="A1:P16"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
@@ -1052,57 +968,57 @@
   <sheetData>
     <row r="1" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A1" s="4" t="s">
-        <v>110</v>
+        <v>82</v>
       </c>
       <c r="B1" s="4" t="s">
-        <v>112</v>
+        <v>84</v>
       </c>
       <c r="C1" s="4" t="s">
-        <v>113</v>
+        <v>85</v>
       </c>
       <c r="D1" s="4" t="s">
-        <v>114</v>
+        <v>86</v>
       </c>
       <c r="E1" s="4" t="s">
-        <v>115</v>
+        <v>87</v>
       </c>
       <c r="F1" s="4" t="s">
-        <v>116</v>
+        <v>88</v>
       </c>
       <c r="G1" s="4" t="s">
-        <v>117</v>
+        <v>89</v>
       </c>
       <c r="H1" s="4" t="s">
-        <v>118</v>
+        <v>90</v>
       </c>
       <c r="I1" s="4" t="s">
-        <v>119</v>
+        <v>91</v>
       </c>
       <c r="J1" s="4" t="s">
-        <v>120</v>
+        <v>92</v>
       </c>
       <c r="K1" s="4" t="s">
-        <v>121</v>
+        <v>93</v>
       </c>
       <c r="L1" s="4" t="s">
-        <v>122</v>
+        <v>94</v>
       </c>
       <c r="M1" s="4" t="s">
-        <v>123</v>
+        <v>95</v>
       </c>
       <c r="N1" s="4" t="s">
-        <v>124</v>
+        <v>96</v>
       </c>
       <c r="O1" s="4" t="s">
-        <v>125</v>
+        <v>97</v>
       </c>
       <c r="P1" s="4" t="s">
-        <v>126</v>
+        <v>98</v>
       </c>
     </row>
     <row r="2" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
-        <v>111</v>
+        <v>83</v>
       </c>
       <c r="B2" s="2">
         <v>2026</v>
@@ -1152,7 +1068,7 @@
     </row>
     <row r="3" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
-        <v>111</v>
+        <v>83</v>
       </c>
       <c r="B3" s="2">
         <v>2027</v>
@@ -1202,7 +1118,7 @@
     </row>
     <row r="4" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
-        <v>111</v>
+        <v>83</v>
       </c>
       <c r="B4" s="2">
         <v>2028</v>
@@ -1252,7 +1168,7 @@
     </row>
     <row r="5" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
-        <v>111</v>
+        <v>83</v>
       </c>
       <c r="B5" s="2">
         <v>2029</v>
@@ -1302,7 +1218,7 @@
     </row>
     <row r="6" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
-        <v>111</v>
+        <v>83</v>
       </c>
       <c r="B6" s="2">
         <v>2030</v>
@@ -1352,7 +1268,7 @@
     </row>
     <row r="7" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
-        <v>127</v>
+        <v>99</v>
       </c>
       <c r="B7" s="2">
         <v>2026</v>
@@ -1402,7 +1318,7 @@
     </row>
     <row r="8" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
-        <v>127</v>
+        <v>99</v>
       </c>
       <c r="B8" s="2">
         <v>2027</v>
@@ -1452,7 +1368,7 @@
     </row>
     <row r="9" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
-        <v>127</v>
+        <v>99</v>
       </c>
       <c r="B9" s="2">
         <v>2028</v>
@@ -1502,7 +1418,7 @@
     </row>
     <row r="10" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
-        <v>127</v>
+        <v>99</v>
       </c>
       <c r="B10" s="2">
         <v>2029</v>
@@ -1552,7 +1468,7 @@
     </row>
     <row r="11" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
-        <v>127</v>
+        <v>99</v>
       </c>
       <c r="B11" s="2">
         <v>2030</v>
@@ -1602,7 +1518,7 @@
     </row>
     <row r="12" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
-        <v>128</v>
+        <v>100</v>
       </c>
       <c r="B12" s="2">
         <v>2026</v>
@@ -1652,7 +1568,7 @@
     </row>
     <row r="13" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
-        <v>128</v>
+        <v>100</v>
       </c>
       <c r="B13" s="2">
         <v>2027</v>
@@ -1702,7 +1618,7 @@
     </row>
     <row r="14" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
-        <v>128</v>
+        <v>100</v>
       </c>
       <c r="B14" s="2">
         <v>2028</v>
@@ -1752,7 +1668,7 @@
     </row>
     <row r="15" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
-        <v>128</v>
+        <v>100</v>
       </c>
       <c r="B15" s="2">
         <v>2029</v>
@@ -1802,7 +1718,7 @@
     </row>
     <row r="16" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
-        <v>128</v>
+        <v>100</v>
       </c>
       <c r="B16" s="2">
         <v>2030</v>
@@ -1856,7 +1772,7 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B6DEF338-C407-4CC7-9F7C-B7EDD0C118AF}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{92D7FE11-2E05-461A-8A4A-B6FC6644F0AB}">
   <dimension ref="A1:E11"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
@@ -1868,24 +1784,24 @@
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A1" s="4" t="s">
-        <v>100</v>
+        <v>72</v>
       </c>
       <c r="B1" s="4" t="s">
-        <v>102</v>
+        <v>74</v>
       </c>
       <c r="C1" s="4" t="s">
-        <v>103</v>
+        <v>75</v>
       </c>
       <c r="D1" s="4" t="s">
-        <v>104</v>
+        <v>76</v>
       </c>
       <c r="E1" s="4" t="s">
-        <v>105</v>
+        <v>77</v>
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
-        <v>101</v>
+        <v>73</v>
       </c>
       <c r="B2" s="5">
         <v>46032</v>
@@ -1902,7 +1818,7 @@
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
-        <v>101</v>
+        <v>73</v>
       </c>
       <c r="B3" s="5">
         <v>46346</v>
@@ -1919,10 +1835,10 @@
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
-        <v>101</v>
+        <v>73</v>
       </c>
       <c r="B4" t="s">
-        <v>106</v>
+        <v>78</v>
       </c>
       <c r="C4" s="2">
         <v>196</v>
@@ -1936,10 +1852,10 @@
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
-        <v>101</v>
+        <v>73</v>
       </c>
       <c r="B5" t="s">
-        <v>107</v>
+        <v>79</v>
       </c>
       <c r="C5" s="2">
         <v>183</v>
@@ -1953,10 +1869,10 @@
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
-        <v>101</v>
+        <v>73</v>
       </c>
       <c r="B6" t="s">
-        <v>108</v>
+        <v>80</v>
       </c>
       <c r="C6" s="2">
         <v>167</v>
@@ -1970,7 +1886,7 @@
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
-        <v>109</v>
+        <v>81</v>
       </c>
       <c r="B7" s="5">
         <v>46032</v>
@@ -1987,7 +1903,7 @@
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
-        <v>109</v>
+        <v>81</v>
       </c>
       <c r="B8" s="5">
         <v>46346</v>
@@ -2004,10 +1920,10 @@
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
-        <v>109</v>
+        <v>81</v>
       </c>
       <c r="B9" t="s">
-        <v>106</v>
+        <v>78</v>
       </c>
       <c r="C9" s="2">
         <v>99</v>
@@ -2021,10 +1937,10 @@
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
-        <v>109</v>
+        <v>81</v>
       </c>
       <c r="B10" t="s">
-        <v>107</v>
+        <v>79</v>
       </c>
       <c r="C10" s="2">
         <v>96</v>
@@ -2038,10 +1954,10 @@
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
-        <v>109</v>
+        <v>81</v>
       </c>
       <c r="B11" t="s">
-        <v>108</v>
+        <v>80</v>
       </c>
       <c r="C11" s="2">
         <v>92</v>
@@ -2059,474 +1975,62 @@
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{938C1E0D-9C19-4C71-B822-BC7949DC9D10}">
-  <dimension ref="A1:C42"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{54923716-118C-44BB-96EE-B8A257373ACA}">
+  <dimension ref="A1:G2"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="7.6640625" bestFit="1" customWidth="1"/>
-    <col min="2" max="3" width="8.5546875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="10.44140625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="10.5546875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="13.77734375" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="255.77734375" bestFit="1" customWidth="1"/>
+    <col min="5" max="6" width="12.6640625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="5.88671875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A1" s="4" t="s">
-        <v>56</v>
+        <v>61</v>
       </c>
       <c r="B1" s="4" t="s">
-        <v>58</v>
+        <v>63</v>
       </c>
       <c r="C1" s="4" t="s">
-        <v>59</v>
-      </c>
-    </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+        <v>64</v>
+      </c>
+      <c r="D1" s="4" t="s">
+        <v>65</v>
+      </c>
+      <c r="E1" s="4" t="s">
+        <v>67</v>
+      </c>
+      <c r="F1" s="4" t="s">
+        <v>69</v>
+      </c>
+      <c r="G1" s="4" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
-        <v>57</v>
-      </c>
-      <c r="B2" s="2">
-        <v>0</v>
-      </c>
-      <c r="C2" s="2">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A3" t="s">
-        <v>60</v>
-      </c>
-      <c r="B3" s="2">
-        <v>0</v>
-      </c>
-      <c r="C3" s="2">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A4" t="s">
-        <v>61</v>
-      </c>
-      <c r="B4" s="2">
-        <v>0</v>
-      </c>
-      <c r="C4" s="2">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A5" t="s">
         <v>62</v>
       </c>
-      <c r="B5" s="2">
-        <v>0</v>
-      </c>
-      <c r="C5" s="2">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A6" t="s">
-        <v>63</v>
-      </c>
-      <c r="B6" s="2">
-        <v>0</v>
-      </c>
-      <c r="C6" s="2">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A7" t="s">
-        <v>64</v>
-      </c>
-      <c r="B7" s="2">
-        <v>0</v>
-      </c>
-      <c r="C7" s="2">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A8" t="s">
-        <v>65</v>
-      </c>
-      <c r="B8" s="2">
-        <v>0</v>
-      </c>
-      <c r="C8" s="2">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A9" t="s">
+      <c r="B2" t="s">
+        <v>62</v>
+      </c>
+      <c r="C2" t="s">
+        <v>62</v>
+      </c>
+      <c r="D2" t="s">
         <v>66</v>
       </c>
-      <c r="B9" s="2">
-        <v>0</v>
-      </c>
-      <c r="C9" s="2">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A10" t="s">
-        <v>67</v>
-      </c>
-      <c r="B10" s="2">
-        <v>0</v>
-      </c>
-      <c r="C10" s="2">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A11" t="s">
+      <c r="E2" t="s">
         <v>68</v>
       </c>
-      <c r="B11" s="2">
-        <v>0</v>
-      </c>
-      <c r="C11" s="2">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A12" t="s">
-        <v>69</v>
-      </c>
-      <c r="B12" s="2">
-        <v>0</v>
-      </c>
-      <c r="C12" s="2">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A13" t="s">
+      <c r="F2" t="s">
         <v>70</v>
       </c>
-      <c r="B13" s="2">
-        <v>0</v>
-      </c>
-      <c r="C13" s="2">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A14" t="s">
-        <v>71</v>
-      </c>
-      <c r="B14" s="2">
-        <v>110000</v>
-      </c>
-      <c r="C14" s="2">
-        <v>160000</v>
-      </c>
-    </row>
-    <row r="15" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A15" t="s">
-        <v>72</v>
-      </c>
-      <c r="B15" s="2">
-        <v>120000</v>
-      </c>
-      <c r="C15" s="2">
-        <v>170000</v>
-      </c>
-    </row>
-    <row r="16" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A16" t="s">
-        <v>73</v>
-      </c>
-      <c r="B16" s="2">
-        <v>130000</v>
-      </c>
-      <c r="C16" s="2">
-        <v>180000</v>
-      </c>
-    </row>
-    <row r="17" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A17" t="s">
-        <v>74</v>
-      </c>
-      <c r="B17" s="2">
-        <v>140000</v>
-      </c>
-      <c r="C17" s="2">
-        <v>190000</v>
-      </c>
-    </row>
-    <row r="18" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A18" t="s">
-        <v>75</v>
-      </c>
-      <c r="B18" s="2">
-        <v>150000</v>
-      </c>
-      <c r="C18" s="2">
-        <v>200000</v>
-      </c>
-    </row>
-    <row r="19" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A19" t="s">
-        <v>76</v>
-      </c>
-      <c r="B19" s="2">
-        <v>160000</v>
-      </c>
-      <c r="C19" s="2">
-        <v>210000</v>
-      </c>
-    </row>
-    <row r="20" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A20" t="s">
-        <v>77</v>
-      </c>
-      <c r="B20" s="2">
-        <v>160000</v>
-      </c>
-      <c r="C20" s="2">
-        <v>901000</v>
-      </c>
-    </row>
-    <row r="21" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A21" t="s">
-        <v>78</v>
-      </c>
-      <c r="B21" s="2">
-        <v>406000</v>
-      </c>
-      <c r="C21" s="2">
-        <v>120000</v>
-      </c>
-    </row>
-    <row r="22" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A22" t="s">
-        <v>79</v>
-      </c>
-      <c r="B22" s="2">
-        <v>120000</v>
-      </c>
-      <c r="C22" s="2">
-        <v>130000</v>
-      </c>
-    </row>
-    <row r="23" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A23" t="s">
-        <v>80</v>
-      </c>
-      <c r="B23" s="2">
-        <v>140000</v>
-      </c>
-      <c r="C23" s="2">
-        <v>145000</v>
-      </c>
-    </row>
-    <row r="24" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A24" t="s">
-        <v>81</v>
-      </c>
-      <c r="B24" s="2">
-        <v>145000</v>
-      </c>
-      <c r="C24" s="2">
-        <v>150000</v>
-      </c>
-    </row>
-    <row r="25" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A25" t="s">
-        <v>82</v>
-      </c>
-      <c r="B25" s="2">
-        <v>150000</v>
-      </c>
-      <c r="C25" s="2">
-        <v>155000</v>
-      </c>
-    </row>
-    <row r="26" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A26" t="s">
-        <v>83</v>
-      </c>
-      <c r="B26" s="2">
-        <v>155000</v>
-      </c>
-      <c r="C26" s="2">
-        <v>160000</v>
-      </c>
-    </row>
-    <row r="27" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A27" t="s">
-        <v>84</v>
-      </c>
-      <c r="B27" s="2">
-        <v>160000</v>
-      </c>
-      <c r="C27" s="2">
-        <v>165000</v>
-      </c>
-    </row>
-    <row r="28" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A28" t="s">
-        <v>85</v>
-      </c>
-      <c r="B28" s="2">
-        <v>165000</v>
-      </c>
-      <c r="C28" s="2">
-        <v>170000</v>
-      </c>
-    </row>
-    <row r="29" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A29" t="s">
-        <v>86</v>
-      </c>
-      <c r="B29" s="2">
-        <v>170000</v>
-      </c>
-      <c r="C29" s="2">
-        <v>175000</v>
-      </c>
-    </row>
-    <row r="30" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A30" t="s">
-        <v>87</v>
-      </c>
-      <c r="B30" s="2">
-        <v>175000</v>
-      </c>
-      <c r="C30" s="2">
-        <v>180000</v>
-      </c>
-    </row>
-    <row r="31" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A31" t="s">
-        <v>88</v>
-      </c>
-      <c r="B31" s="2">
-        <v>180000</v>
-      </c>
-      <c r="C31" s="2">
-        <v>185000</v>
-      </c>
-    </row>
-    <row r="32" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A32" t="s">
-        <v>89</v>
-      </c>
-      <c r="B32" s="2">
-        <v>185000</v>
-      </c>
-      <c r="C32" s="2">
-        <v>190000</v>
-      </c>
-    </row>
-    <row r="33" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A33" t="s">
-        <v>90</v>
-      </c>
-      <c r="B33" s="2">
-        <v>190000</v>
-      </c>
-      <c r="C33" s="2">
-        <v>195000</v>
-      </c>
-    </row>
-    <row r="34" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A34" t="s">
-        <v>91</v>
-      </c>
-      <c r="B34" s="2">
-        <v>195000</v>
-      </c>
-      <c r="C34" s="2">
-        <v>200000</v>
-      </c>
-    </row>
-    <row r="35" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A35" t="s">
-        <v>92</v>
-      </c>
-      <c r="B35" s="2">
-        <v>200000</v>
-      </c>
-      <c r="C35" s="2">
-        <v>205000</v>
-      </c>
-    </row>
-    <row r="36" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A36" t="s">
-        <v>93</v>
-      </c>
-      <c r="B36" s="2">
-        <v>205000</v>
-      </c>
-      <c r="C36" s="2">
-        <v>210000</v>
-      </c>
-    </row>
-    <row r="37" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A37" t="s">
-        <v>94</v>
-      </c>
-      <c r="B37" s="2">
-        <v>210000</v>
-      </c>
-      <c r="C37" s="2">
-        <v>215000</v>
-      </c>
-    </row>
-    <row r="38" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A38" t="s">
-        <v>95</v>
-      </c>
-      <c r="B38" s="2">
-        <v>215000</v>
-      </c>
-      <c r="C38" s="2">
-        <v>220000</v>
-      </c>
-    </row>
-    <row r="39" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A39" t="s">
-        <v>96</v>
-      </c>
-      <c r="B39" s="2">
-        <v>220000</v>
-      </c>
-      <c r="C39" s="2">
-        <v>225000</v>
-      </c>
-    </row>
-    <row r="40" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A40" t="s">
-        <v>97</v>
-      </c>
-      <c r="B40" s="2">
-        <v>225000</v>
-      </c>
-      <c r="C40" s="2">
-        <v>230000</v>
-      </c>
-    </row>
-    <row r="41" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A41" t="s">
-        <v>98</v>
-      </c>
-      <c r="B41" s="2">
-        <v>230000</v>
-      </c>
-      <c r="C41" s="2">
-        <v>235000</v>
-      </c>
-    </row>
-    <row r="42" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A42" t="s">
-        <v>99</v>
-      </c>
-      <c r="B42" s="2">
-        <v>235000</v>
-      </c>
-      <c r="C42" s="2">
-        <v>240000</v>
+      <c r="G2" s="2">
+        <v>36</v>
       </c>
     </row>
   </sheetData>
@@ -2535,12 +2039,12 @@
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B141AFE5-B7B8-4317-B3FC-9A9AE8886C9F}">
-  <dimension ref="A1:B8"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9C734D11-BD48-45D4-896E-9720F449DE57}">
+  <dimension ref="A1:B11"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="14" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="38.21875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="17.21875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="58.77734375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.3">
@@ -2553,7 +2057,7 @@
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="B2" s="1">
         <v>46265</v>
@@ -2561,49 +2065,73 @@
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="B3" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="B4" s="2">
-        <v>803</v>
+        <v>34</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="B5" s="2">
-        <v>172</v>
+        <v>803</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="B6" s="2">
-        <v>963</v>
+        <v>172</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="B7" s="2">
-        <v>4512</v>
+        <v>4</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="B8" s="2">
+        <v>963</v>
+      </c>
+    </row>
+    <row r="9" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A9" t="s">
+        <v>58</v>
+      </c>
+      <c r="B9" s="2">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="10" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A10" t="s">
+        <v>59</v>
+      </c>
+      <c r="B10" s="2">
+        <v>4512</v>
+      </c>
+    </row>
+    <row r="11" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A11" t="s">
+        <v>60</v>
+      </c>
+      <c r="B11" s="2">
         <v>3422</v>
       </c>
     </row>
@@ -2613,8 +2141,8 @@
 </file>
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{781BD633-0532-46F8-AB61-E47D0A3BFBAD}">
-  <dimension ref="A1:B24"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E1FFB593-0D81-4582-853B-B0B6B2E57672}">
+  <dimension ref="A1:B26"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="23.88671875" bestFit="1" customWidth="1"/>
@@ -2650,7 +2178,7 @@
         <v>26</v>
       </c>
       <c r="B4" s="2">
-        <v>1800</v>
+        <v>800</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.3">
@@ -2658,7 +2186,7 @@
         <v>27</v>
       </c>
       <c r="B5" s="2">
-        <v>1200</v>
+        <v>800</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.3">
@@ -2666,7 +2194,7 @@
         <v>28</v>
       </c>
       <c r="B6" s="2">
-        <v>250</v>
+        <v>1800</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.3">
@@ -2674,7 +2202,7 @@
         <v>29</v>
       </c>
       <c r="B7" s="2">
-        <v>150</v>
+        <v>1200</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.3">
@@ -2682,7 +2210,7 @@
         <v>30</v>
       </c>
       <c r="B8" s="2">
-        <v>400</v>
+        <v>250</v>
       </c>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.3">
@@ -2690,7 +2218,7 @@
         <v>31</v>
       </c>
       <c r="B9" s="2">
-        <v>0.03</v>
+        <v>150</v>
       </c>
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.3">
@@ -2698,7 +2226,7 @@
         <v>32</v>
       </c>
       <c r="B10" s="2">
-        <v>0.05</v>
+        <v>400</v>
       </c>
     </row>
     <row r="11" spans="1:2" x14ac:dyDescent="0.3">
@@ -2706,7 +2234,7 @@
         <v>33</v>
       </c>
       <c r="B11" s="2">
-        <v>0.08</v>
+        <v>0.03</v>
       </c>
     </row>
     <row r="12" spans="1:2" x14ac:dyDescent="0.3">
@@ -2714,7 +2242,7 @@
         <v>34</v>
       </c>
       <c r="B12" s="2">
-        <v>0.2</v>
+        <v>0.05</v>
       </c>
     </row>
     <row r="13" spans="1:2" x14ac:dyDescent="0.3">
@@ -2722,7 +2250,7 @@
         <v>35</v>
       </c>
       <c r="B13" s="2">
-        <v>3</v>
+        <v>0.08</v>
       </c>
     </row>
     <row r="14" spans="1:2" x14ac:dyDescent="0.3">
@@ -2730,7 +2258,7 @@
         <v>36</v>
       </c>
       <c r="B14" s="2">
-        <v>1</v>
+        <v>0.2</v>
       </c>
     </row>
     <row r="15" spans="1:2" x14ac:dyDescent="0.3">
@@ -2738,7 +2266,7 @@
         <v>37</v>
       </c>
       <c r="B15" s="2">
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="16" spans="1:2" x14ac:dyDescent="0.3">
@@ -2746,31 +2274,31 @@
         <v>38</v>
       </c>
       <c r="B16" s="2">
-        <v>0.6</v>
+        <v>1</v>
       </c>
     </row>
     <row r="17" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
         <v>39</v>
       </c>
-      <c r="B17" t="s">
-        <v>40</v>
+      <c r="B17" s="2">
+        <v>1</v>
       </c>
     </row>
     <row r="18" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A18" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="B18" s="2">
-        <v>600</v>
+        <v>0.6</v>
       </c>
     </row>
     <row r="19" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A19" t="s">
+        <v>41</v>
+      </c>
+      <c r="B19" t="s">
         <v>42</v>
-      </c>
-      <c r="B19" s="2">
-        <v>0.3</v>
       </c>
     </row>
     <row r="20" spans="1:2" x14ac:dyDescent="0.3">
@@ -2778,7 +2306,7 @@
         <v>43</v>
       </c>
       <c r="B20" s="2">
-        <v>600000</v>
+        <v>600</v>
       </c>
     </row>
     <row r="21" spans="1:2" x14ac:dyDescent="0.3">
@@ -2786,7 +2314,7 @@
         <v>44</v>
       </c>
       <c r="B21" s="2">
-        <v>96</v>
+        <v>0.3</v>
       </c>
     </row>
     <row r="22" spans="1:2" x14ac:dyDescent="0.3">
@@ -2794,7 +2322,7 @@
         <v>45</v>
       </c>
       <c r="B22" s="2">
-        <v>60</v>
+        <v>600000</v>
       </c>
     </row>
     <row r="23" spans="1:2" x14ac:dyDescent="0.3">
@@ -2802,7 +2330,7 @@
         <v>46</v>
       </c>
       <c r="B23" s="2">
-        <v>36000</v>
+        <v>96</v>
       </c>
     </row>
     <row r="24" spans="1:2" x14ac:dyDescent="0.3">
@@ -2810,6 +2338,22 @@
         <v>47</v>
       </c>
       <c r="B24" s="2">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="25" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A25" t="s">
+        <v>48</v>
+      </c>
+      <c r="B25" s="2">
+        <v>36000</v>
+      </c>
+    </row>
+    <row r="26" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A26" t="s">
+        <v>49</v>
+      </c>
+      <c r="B26" s="2">
         <v>5.7</v>
       </c>
     </row>
@@ -2819,12 +2363,12 @@
 </file>
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D72A9D5C-27BE-4279-9322-10D3885C563B}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A3E148F8-3DFE-42C2-BEF9-08BE1FBD215E}">
   <dimension ref="A1:B22"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="32.33203125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="10.33203125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="11.5546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.3">
@@ -2872,7 +2416,7 @@
         <v>6</v>
       </c>
       <c r="B6" s="2">
-        <v>5786400</v>
+        <v>5396400</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.3">
@@ -2888,7 +2432,7 @@
         <v>8</v>
       </c>
       <c r="B8" s="2">
-        <v>2008512</v>
+        <v>1618512</v>
       </c>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.3">
@@ -2896,7 +2440,7 @@
         <v>9</v>
       </c>
       <c r="B9" s="3">
-        <v>0.65290000000000004</v>
+        <v>0.70009999999999994</v>
       </c>
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.3">
@@ -2904,7 +2448,7 @@
         <v>10</v>
       </c>
       <c r="B10" s="2">
-        <v>2070000</v>
+        <v>2008247.07</v>
       </c>
     </row>
     <row r="11" spans="1:2" x14ac:dyDescent="0.3">
@@ -3009,7 +2553,7 @@
 </file>
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AD300348-C963-45E1-B61E-2D95C7F779CA}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8EAB1686-7CE9-4932-872F-52640B2E0C0C}">
   <dimension ref="A1"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData/>

</xml_diff>